<commit_message>
Fix submission scoring and clean artifacts
</commit_message>
<xml_diff>
--- a/submission/redrob_ranked_output.xlsx
+++ b/submission/redrob_ranked_output.xlsx
@@ -108,7 +108,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer with 7.0 yrs; career evidence includes semantic search, embeddings, and retrieval system; Kochi, Kerala; response rate 0.95; notice 60 days.</t>
+          <t>Staff Machine Learning Engineer shortlisted for strong role fit in BM25 retrieval, Information Retrieval, and LLM systems; fit 100, proof 77, confidence 100, risk 0; Kochi, Kerala; strong availability signals.</t>
         </is>
       </c>
     </row>
@@ -122,11 +122,11 @@
         <v>2</v>
       </c>
       <c r="C3" s="2">
-        <v>0.9801</v>
+        <v>0.9895</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Senior Machine Learning Engineer with 7.2 yrs; career evidence includes embeddings, faiss, and retrieval system; Noida, Uttar Pradesh; response rate 0.61; notice 15 days.</t>
+          <t>Senior Machine Learning Engineer shortlisted for strong role fit in BM25 retrieval, Embeddings, and Information Retrieval; fit 100, proof 78, confidence 100, risk 0; Noida, Uttar Pradesh; strong availability signals; good logistics fit.</t>
         </is>
       </c>
     </row>
@@ -140,11 +140,11 @@
         <v>3</v>
       </c>
       <c r="C4" s="2">
-        <v>0.9702</v>
+        <v>0.9334</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer with 8.6 yrs; career evidence includes embeddings, pinecone, and retrieval system; Jaipur, Rajasthan; response rate 0.83; notice 90 days.</t>
+          <t>Staff Machine Learning Engineer shortlisted for strong role fit in BM25 retrieval, Elasticsearch, and Hugging Face Transformers; fit 100, proof 74, confidence 100, risk 0; Jaipur, Rajasthan; strong availability signals.</t>
         </is>
       </c>
     </row>
@@ -158,11 +158,11 @@
         <v>4</v>
       </c>
       <c r="C5" s="2">
-        <v>0.9603</v>
+        <v>0.9199</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Lead AI Engineer with 6.7 yrs; career evidence includes semantic search, embeddings, and vector search; Jaipur, Rajasthan; response rate 0.73; notice 30 days.</t>
+          <t>Lead AI Engineer shortlisted for strong role fit in BM25 retrieval, Elasticsearch, and Embeddings; fit 100, proof 62, confidence 100, risk 0; Jaipur, Rajasthan; strong availability signals.</t>
         </is>
       </c>
     </row>
@@ -176,11 +176,11 @@
         <v>5</v>
       </c>
       <c r="C6" s="2">
-        <v>0.9504</v>
+        <v>0.9046</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Senior AI Engineer with 7.8 yrs; career evidence includes embeddings, pinecone, and recommendation system; Vizag, Andhra Pradesh; response rate 0.76; notice 45 days.</t>
+          <t>Senior AI Engineer shortlisted for strong role fit in BM25 retrieval, Elasticsearch, and Embeddings; fit 100, proof 71, confidence 100, risk 0; Vizag, Andhra Pradesh; strong availability signals.</t>
         </is>
       </c>
     </row>
@@ -194,11 +194,11 @@
         <v>6</v>
       </c>
       <c r="C7" s="2">
-        <v>0.9405</v>
+        <v>0.8868</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Senior NLP Engineer with 8.9 yrs; career evidence includes embeddings, vector search, and faiss; Coimbatore, Tamil Nadu; response rate 0.78; notice 30 days.</t>
+          <t>Senior NLP Engineer shortlisted for strong role fit in BM25 retrieval, Elasticsearch, and OpenSearch; fit 98, proof 70, confidence 100, risk 0; Coimbatore, Tamil Nadu; strong availability signals.</t>
         </is>
       </c>
     </row>
@@ -212,11 +212,11 @@
         <v>7</v>
       </c>
       <c r="C8" s="2">
-        <v>0.9306</v>
+        <v>0.8800</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Applied ML Engineer with 8.0 yrs; career evidence includes embeddings, pinecone, and relevance systems; Pune, Maharashtra; response rate 0.42; notice 30 days.</t>
+          <t>Applied ML Engineer shortlisted for strong role fit in Embeddings, OpenSearch, and Pinecone; fit 89, proof 65, confidence 100, risk 0; Pune, Maharashtra; strong availability signals; good logistics fit.</t>
         </is>
       </c>
     </row>
@@ -230,11 +230,11 @@
         <v>8</v>
       </c>
       <c r="C9" s="2">
-        <v>0.9207</v>
+        <v>0.8795</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Senior AI Engineer with 7.9 yrs; career evidence includes search and discovery, matching layer, and relevance systems; Noida, Uttar Pradesh; response rate 0.79; notice 60 days.</t>
+          <t>Senior AI Engineer shortlisted for strong role fit in BM25 retrieval, Kubernetes, and NLP; fit 99, proof 53, confidence 100, risk 0; Noida, Uttar Pradesh; strong availability signals; good logistics fit.</t>
         </is>
       </c>
     </row>
@@ -248,11 +248,11 @@
         <v>9</v>
       </c>
       <c r="C10" s="2">
-        <v>0.9108</v>
+        <v>0.8769</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Search Engineer with 7.6 yrs; career evidence includes embeddings, pinecone, and relevance systems; Gurgaon, Haryana; response rate 0.94; notice 45 days.</t>
+          <t>Search Engineer shortlisted for strong role fit in BM25 retrieval, Milvus, and PyTorch; fit 94, proof 59, confidence 100, risk 0; Gurgaon, Haryana; strong availability signals; good logistics fit.</t>
         </is>
       </c>
     </row>
@@ -266,11 +266,11 @@
         <v>10</v>
       </c>
       <c r="C11" s="2">
-        <v>0.9009</v>
+        <v>0.8696</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer with 8.0 yrs; career evidence includes embeddings, pinecone, and relevance systems; Noida, Uttar Pradesh; response rate 0.77; notice 60 days.</t>
+          <t>Recommendation Systems Engineer shortlisted for strong role fit in FAISS/vector search, Information Retrieval, and MLOps; fit 92, proof 56, confidence 100, risk 0; Noida, Uttar Pradesh; strong availability signals; good logistics fit.</t>
         </is>
       </c>
     </row>
@@ -284,11 +284,11 @@
         <v>11</v>
       </c>
       <c r="C12" s="2">
-        <v>0.8910</v>
+        <v>0.8652</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Senior Machine Learning Engineer with 6.1 yrs; career evidence includes embeddings, faiss, and retrieval system; Pune, Maharashtra; response rate 0.88; notice 60 days.</t>
+          <t>Senior Machine Learning Engineer shortlisted for strong role fit in Elasticsearch, Information Retrieval, and LLM systems; fit 93, proof 56, confidence 90, risk 0; Pune, Maharashtra; strong availability signals; good logistics fit.</t>
         </is>
       </c>
     </row>
@@ -302,11 +302,11 @@
         <v>12</v>
       </c>
       <c r="C13" s="2">
-        <v>0.8811</v>
+        <v>0.8610</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Senior Applied Scientist with 5.3 yrs; career evidence includes embeddings, vector search, and faiss; Kolkata, West Bengal; response rate 0.55; notice 0 days.</t>
+          <t>Senior Applied Scientist shortlisted for strong role fit in Elasticsearch, Embeddings, and Fine-tuning LLMs; fit 94, proof 61, confidence 100, risk 0; Kolkata, West Bengal; strong availability signals; good logistics fit.</t>
         </is>
       </c>
     </row>
@@ -320,11 +320,11 @@
         <v>13</v>
       </c>
       <c r="C14" s="2">
-        <v>0.8712</v>
+        <v>0.8567</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer with 6.0 yrs; career evidence includes embeddings, relevance systems, and ranking; Hyderabad, Telangana; response rate 0.91; notice 60 days.</t>
+          <t>Recommendation Systems Engineer shortlisted for strong role fit in BentoML, Embeddings, and FAISS/vector search; fit 90, proof 61, confidence 100, risk 0; Hyderabad, Telangana; strong availability signals; good logistics fit.</t>
         </is>
       </c>
     </row>
@@ -338,11 +338,11 @@
         <v>14</v>
       </c>
       <c r="C15" s="2">
-        <v>0.8613</v>
+        <v>0.8512</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>AI Engineer with 6.9 yrs; career evidence includes semantic search, embeddings, and faiss; Trivandrum, Kerala; response rate 0.81; notice 30 days.</t>
+          <t>AI Engineer shortlisted for strong role fit in BM25 retrieval, BentoML, and Learning to Rank; fit 85, proof 64, confidence 100, risk 0; Trivandrum, Kerala; strong availability signals.</t>
         </is>
       </c>
     </row>
@@ -356,11 +356,11 @@
         <v>15</v>
       </c>
       <c r="C16" s="2">
-        <v>0.8514</v>
+        <v>0.8498</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer with 6.7 yrs; career evidence includes embeddings, pinecone, and relevance systems; Indore, Madhya Pradesh; response rate 0.52; notice 30 days.</t>
+          <t>Recommendation Systems Engineer shortlisted for strong role fit in BM25 retrieval, Elasticsearch, and Embeddings; fit 85, proof 55, confidence 100, risk 0; Indore, Madhya Pradesh; strong availability signals; verify evaluation methodology or ranking metrics.</t>
         </is>
       </c>
     </row>
@@ -374,11 +374,11 @@
         <v>16</v>
       </c>
       <c r="C17" s="2">
-        <v>0.8415</v>
+        <v>0.8382</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Applied ML Engineer with 7.4 yrs; career evidence includes embeddings, pinecone, and relevance systems; Noida, Uttar Pradesh; response rate 0.76; notice 120 days. Concern: long notice period.</t>
+          <t>Applied ML Engineer shortlisted for strong role fit in BM25 retrieval, Milvus, and Pinecone; fit 89, proof 64, confidence 100, risk 10; Noida, Uttar Pradesh; strong availability signals; good logistics fit; verify Notice period may slow hiring.</t>
         </is>
       </c>
     </row>
@@ -392,11 +392,11 @@
         <v>17</v>
       </c>
       <c r="C18" s="2">
-        <v>0.8316</v>
+        <v>0.8343</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Senior Applied Scientist with 16.2 yrs; career evidence includes semantic search, embeddings, and faiss; Indore, Madhya Pradesh; response rate 0.81; notice 30 days.</t>
+          <t>Senior Applied Scientist shortlisted for strong role fit in BM25 retrieval, Elasticsearch, and Fine-tuning LLMs; fit 99, proof 84, confidence 100, risk 16; Indore, Madhya Pradesh; strong availability signals; good logistics fit.</t>
         </is>
       </c>
     </row>
@@ -410,11 +410,11 @@
         <v>18</v>
       </c>
       <c r="C19" s="2">
-        <v>0.8217</v>
+        <v>0.8304</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Applied ML Engineer with 6.0 yrs; career evidence includes embeddings, relevance systems, and recommendation system; Kolkata, West Bengal; response rate 0.67; notice 90 days.</t>
+          <t>Applied ML Engineer shortlisted for strong role fit in FAISS/vector search, MLOps, and Machine Learning; fit 91, proof 63, confidence 100, risk 0; Kolkata, West Bengal; strong availability signals.</t>
         </is>
       </c>
     </row>
@@ -428,11 +428,11 @@
         <v>19</v>
       </c>
       <c r="C20" s="2">
-        <v>0.8118</v>
+        <v>0.8294</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Senior NLP Engineer with 7.8 yrs; career evidence includes semantic search, embeddings, and pinecone; Kolkata, West Bengal; response rate 0.66; notice 90 days.</t>
+          <t>Senior NLP Engineer shortlisted for strong role fit in Hugging Face Transformers, Information Retrieval, and Learning to Rank; fit 88, proof 63, confidence 100, risk 0; Kolkata, West Bengal; strong availability signals.</t>
         </is>
       </c>
     </row>
@@ -446,11 +446,11 @@
         <v>20</v>
       </c>
       <c r="C21" s="2">
-        <v>0.8019</v>
+        <v>0.8191</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 7.4 yrs; career evidence includes semantic search, embeddings, and faiss; Delhi, Delhi; response rate 0.57; notice 90 days.</t>
+          <t>Senior Data Scientist shortlisted for strong role fit in Fine-tuning LLMs, Information Retrieval, and RAG; fit 80, proof 54, confidence 100, risk 0; Delhi, Delhi; strong availability signals; good logistics fit.</t>
         </is>
       </c>
     </row>
@@ -464,11 +464,11 @@
         <v>21</v>
       </c>
       <c r="C22" s="2">
-        <v>0.7920</v>
+        <v>0.8170</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer with 7.7 yrs; career evidence includes semantic search, embeddings, and faiss; Bangalore, Karnataka; response rate 0.72; notice 60 days.</t>
+          <t>Recommendation Systems Engineer shortlisted for strong role fit in BentoML, Hugging Face Transformers, and Information Retrieval; fit 85, proof 48, confidence 99, risk 0; Bangalore, Karnataka; strong availability signals; good logistics fit.</t>
         </is>
       </c>
     </row>
@@ -482,11 +482,11 @@
         <v>22</v>
       </c>
       <c r="C23" s="2">
-        <v>0.7821</v>
+        <v>0.8136</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Search Engineer with 7.8 yrs; career evidence includes embeddings, pinecone, and relevance systems; Kolkata, West Bengal; response rate 0.58; notice 90 days.</t>
+          <t>Search Engineer shortlisted for strong role fit in BM25 retrieval, BentoML, and Elasticsearch; fit 88, proof 55, confidence 100, risk 0; Kolkata, West Bengal; strong availability signals.</t>
         </is>
       </c>
     </row>
@@ -500,11 +500,11 @@
         <v>23</v>
       </c>
       <c r="C24" s="2">
-        <v>0.7722</v>
+        <v>0.8103</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>AI Engineer with 7.6 yrs; career evidence includes embeddings, pinecone, and relevance systems; Indore, Madhya Pradesh; response rate 0.62; notice 45 days.</t>
+          <t>AI Engineer shortlisted for strong role fit in BentoML, Hugging Face Transformers, and MLOps; fit 77, proof 51, confidence 99, risk 0; Indore, Madhya Pradesh; strong availability signals; good logistics fit; verify evaluation methodology or ranking metrics.</t>
         </is>
       </c>
     </row>
@@ -518,11 +518,11 @@
         <v>24</v>
       </c>
       <c r="C25" s="2">
-        <v>0.7623</v>
+        <v>0.8101</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 7.8 yrs; career evidence includes embeddings, relevance systems, and recommendation system; Trivandrum, Kerala; response rate 0.48; notice 15 days.</t>
+          <t>Senior Data Scientist shortlisted for strong role fit in Fine-tuning LLMs, MLflow, and Machine Learning; fit 89, proof 68, confidence 100, risk 1; Trivandrum, Kerala.</t>
         </is>
       </c>
     </row>
@@ -536,11 +536,11 @@
         <v>25</v>
       </c>
       <c r="C26" s="2">
-        <v>0.7524</v>
+        <v>0.8099</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Applied ML Engineer with 6.2 yrs; career evidence includes semantic search, embeddings, and faiss; Indore, Madhya Pradesh; response rate 0.64; notice 120 days. Concern: long notice period.</t>
+          <t>Applied ML Engineer shortlisted for strong role fit in BentoML, FAISS/vector search, and Fine-tuning LLMs; fit 93, proof 72, confidence 100, risk 10; Indore, Madhya Pradesh; verify Notice period may slow hiring.</t>
         </is>
       </c>
     </row>
@@ -554,11 +554,11 @@
         <v>26</v>
       </c>
       <c r="C27" s="2">
-        <v>0.7425</v>
+        <v>0.8088</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Search Engineer with 7.8 yrs; career evidence includes semantic search, embeddings, and faiss; Chennai, Tamil Nadu; response rate 0.63; notice 45 days. Concern: not marked open to work.</t>
+          <t>Search Engineer shortlisted for strong role fit in Hugging Face Transformers, Learning to Rank, and MLOps; fit 100, proof 75, confidence 100, risk 28; Chennai, Tamil Nadu; verify Availability is weaker because the candidate is not marked open to work.</t>
         </is>
       </c>
     </row>
@@ -572,11 +572,11 @@
         <v>27</v>
       </c>
       <c r="C28" s="2">
-        <v>0.7326</v>
+        <v>0.8065</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer with 8.8 yrs; career evidence includes semantic search, embeddings, and search and discovery; Coimbatore, Tamil Nadu; response rate 0.66; notice 0 days. Concern: not marked open to work.</t>
+          <t>Staff Machine Learning Engineer shortlisted for strong role fit in Elasticsearch, Information Retrieval Systems, and LoRA; fit 96, proof 61, confidence 100, risk 28; Coimbatore, Tamil Nadu; strong availability signals; good logistics fit; verify Availability is weaker because the candidate is not marked open to work.</t>
         </is>
       </c>
     </row>
@@ -590,11 +590,11 @@
         <v>28</v>
       </c>
       <c r="C29" s="2">
-        <v>0.7227</v>
+        <v>0.8056</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Senior AI Engineer with 5.9 yrs; career evidence includes embeddings, matching layer, and relevance systems; Kolkata, West Bengal; response rate 0.81; notice 90 days.</t>
+          <t>Senior AI Engineer shortlisted for strong role fit in Information Retrieval Systems, LoRA, and PyTorch; fit 93, proof 51, confidence 97, risk 0; Kolkata, West Bengal; strong availability signals.</t>
         </is>
       </c>
     </row>
@@ -608,11 +608,11 @@
         <v>29</v>
       </c>
       <c r="C30" s="2">
-        <v>0.7128</v>
+        <v>0.8035</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Search Engineer with 5.2 yrs; career evidence includes embeddings, recommendation system, and ranking; Chennai, Tamil Nadu; response rate 0.46; notice 30 days.</t>
+          <t>Search Engineer shortlisted for strong role fit in Airflow, FAISS/vector search, and LoRA; fit 90, proof 55, confidence 100, risk 0; Chennai, Tamil Nadu.</t>
         </is>
       </c>
     </row>
@@ -626,11 +626,11 @@
         <v>30</v>
       </c>
       <c r="C31" s="2">
-        <v>0.7029</v>
+        <v>0.7994</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Applied ML Engineer with 7.1 yrs; career evidence includes semantic search, faiss, and elasticsearch; Gurgaon, Haryana; response rate 0.61; notice 90 days.</t>
+          <t>Applied ML Engineer shortlisted for strong role fit in Elasticsearch, FAISS/vector search, and Hugging Face Transformers; fit 85, proof 48, confidence 100, risk 0; Gurgaon, Haryana; strong availability signals; good logistics fit.</t>
         </is>
       </c>
     </row>
@@ -644,11 +644,11 @@
         <v>31</v>
       </c>
       <c r="C32" s="2">
-        <v>0.6930</v>
+        <v>0.7985</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Senior AI Engineer with 5.9 yrs; career evidence includes embeddings, retrieval system, and recommendation system; Trivandrum, Kerala; response rate 0.80; notice 30 days.</t>
+          <t>Senior AI Engineer shortlisted for strong role fit in FAISS/vector search, Fine-tuning LLMs, and NLP; fit 81, proof 47, confidence 100, risk 0; Trivandrum, Kerala; strong availability signals.</t>
         </is>
       </c>
     </row>
@@ -662,11 +662,11 @@
         <v>32</v>
       </c>
       <c r="C33" s="2">
-        <v>0.6831</v>
+        <v>0.7961</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>NLP Engineer with 6.7 yrs; career evidence includes semantic search, faiss, and elasticsearch; Kolkata, West Bengal; response rate 0.83; notice 30 days.</t>
+          <t>NLP Engineer shortlisted for strong role fit in Elasticsearch, Information Retrieval, and MLflow; fit 83, proof 57, confidence 93, risk 1; Kolkata, West Bengal; strong availability signals.</t>
         </is>
       </c>
     </row>
@@ -680,11 +680,11 @@
         <v>33</v>
       </c>
       <c r="C34" s="2">
-        <v>0.6732</v>
+        <v>0.7951</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer with 5.8 yrs; career evidence includes embeddings, relevance systems, and ranking; Coimbatore, Tamil Nadu; response rate 0.75; notice 90 days.</t>
+          <t>Recommendation Systems Engineer shortlisted for strong role fit in Embeddings, FAISS/vector search, and LoRA; fit 81, proof 45, confidence 94, risk 0; Coimbatore, Tamil Nadu; strong availability signals; good logistics fit.</t>
         </is>
       </c>
     </row>
@@ -698,11 +698,11 @@
         <v>34</v>
       </c>
       <c r="C35" s="2">
-        <v>0.6633</v>
+        <v>0.7924</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer with 7.7 yrs; career evidence includes semantic search, embeddings, and faiss; Vizag, Andhra Pradesh; response rate 0.52; notice 120 days. Concern: long notice period.</t>
+          <t>Recommendation Systems Engineer shortlisted for strong role fit in BM25 retrieval, BentoML, and Elasticsearch; fit 92, proof 57, confidence 100, risk 10; Vizag, Andhra Pradesh; verify Notice period may slow hiring.</t>
         </is>
       </c>
     </row>
@@ -716,11 +716,11 @@
         <v>35</v>
       </c>
       <c r="C36" s="2">
-        <v>0.6534</v>
+        <v>0.7894</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Search Engineer with 4.2 yrs; career evidence includes embeddings, recommendation system, and ranking; Chandigarh, Chandigarh; response rate 0.90; notice 90 days.</t>
+          <t>Search Engineer shortlisted for strong role fit in BentoML, Information Retrieval, and LLM systems; fit 85, proof 59, confidence 97, risk 0; Chandigarh, Chandigarh.</t>
         </is>
       </c>
     </row>
@@ -734,11 +734,11 @@
         <v>36</v>
       </c>
       <c r="C37" s="2">
-        <v>0.6435</v>
+        <v>0.7864</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Search Engineer with 7.8 yrs; career evidence includes semantic search, embeddings, and faiss; Vizag, Andhra Pradesh; response rate 0.70; notice 120 days. Concern: long notice period.</t>
+          <t>Search Engineer shortlisted for strong role fit in Embeddings, Learning to Rank, and MLflow; fit 87, proof 59, confidence 100, risk 10; Vizag, Andhra Pradesh; strong availability signals; verify Notice period may slow hiring.</t>
         </is>
       </c>
     </row>
@@ -752,11 +752,11 @@
         <v>37</v>
       </c>
       <c r="C38" s="2">
-        <v>0.6336</v>
+        <v>0.7849</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Applied ML Engineer with 6.6 yrs; career evidence includes semantic search, embeddings, and faiss; Bhubaneswar, Odisha; response rate 0.78; notice 90 days.</t>
+          <t>Applied ML Engineer shortlisted for strong role fit in Hugging Face Transformers, Learning to Rank, and LoRA; fit 82, proof 48, confidence 85, risk 0; Bhubaneswar, Odisha; strong availability signals; good logistics fit; verify career-backed ranking proof.</t>
         </is>
       </c>
     </row>
@@ -770,11 +770,11 @@
         <v>38</v>
       </c>
       <c r="C39" s="2">
-        <v>0.6237</v>
+        <v>0.7829</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer with 6.3 yrs; career evidence includes embeddings, recommendation system, and ranking; Coimbatore, Tamil Nadu; response rate 0.86; notice 60 days.</t>
+          <t>Machine Learning Engineer shortlisted for strong role fit in BentoML, FastAPI, and Hugging Face Transformers; fit 84, proof 57, confidence 95, risk 0; Coimbatore, Tamil Nadu; strong availability signals.</t>
         </is>
       </c>
     </row>
@@ -788,11 +788,11 @@
         <v>39</v>
       </c>
       <c r="C40" s="2">
-        <v>0.6138</v>
+        <v>0.7768</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer with 6.4 yrs; career evidence includes embeddings, relevance systems, and ranking; Chennai, Tamil Nadu; response rate 0.64; notice 60 days.</t>
+          <t>Recommendation Systems Engineer shortlisted for strong role fit in Elasticsearch, FAISS/vector search, and Fine-tuning LLMs; fit 82, proof 47, confidence 81, risk 0; Chennai, Tamil Nadu; strong availability signals; verify evaluation methodology or ranking metrics.</t>
         </is>
       </c>
     </row>
@@ -806,11 +806,11 @@
         <v>40</v>
       </c>
       <c r="C41" s="2">
-        <v>0.6039</v>
+        <v>0.7732</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>AI Engineer with 6.8 yrs; career evidence includes semantic search, embeddings, and faiss; Delhi, Delhi; response rate 0.77; notice 30 days.</t>
+          <t>AI Engineer shortlisted for strong role fit in BM25 retrieval, FAISS/vector search, and Fine-tuning LLMs; fit 83, proof 49, confidence 85, risk 1; Delhi, Delhi; strong availability signals; good logistics fit; verify evaluation methodology or ranking metrics.</t>
         </is>
       </c>
     </row>
@@ -824,11 +824,11 @@
         <v>41</v>
       </c>
       <c r="C42" s="2">
-        <v>0.5940</v>
+        <v>0.7713</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Senior NLP Engineer with 7.8 yrs; career evidence includes embeddings, pinecone, and recommendations; Indore, Madhya Pradesh; response rate 0.89; notice 15 days.</t>
+          <t>Senior NLP Engineer shortlisted for strong role fit in Embeddings, FAISS/vector search, and MLOps; fit 83, proof 50, confidence 88, risk 0; Indore, Madhya Pradesh; strong availability signals.</t>
         </is>
       </c>
     </row>
@@ -842,11 +842,11 @@
         <v>42</v>
       </c>
       <c r="C43" s="2">
-        <v>0.5841</v>
+        <v>0.7673</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Search Engineer with 7.2 yrs; career evidence includes semantic search, embeddings, and faiss; Trivandrum, Kerala; response rate 0.57; notice 120 days. Concern: long notice period.</t>
+          <t>Search Engineer shortlisted for strong role fit in Embeddings, Information Retrieval, and Learning to Rank; fit 87, proof 47, confidence 97, risk 10; Trivandrum, Kerala; strong availability signals; good logistics fit; verify Notice period may slow hiring.</t>
         </is>
       </c>
     </row>
@@ -860,11 +860,11 @@
         <v>43</v>
       </c>
       <c r="C44" s="2">
-        <v>0.5742</v>
+        <v>0.7657</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer with 5.8 yrs; career evidence includes semantic search, faiss, and elasticsearch; Bhubaneswar, Odisha; response rate 0.60; notice 15 days.</t>
+          <t>Recommendation Systems Engineer shortlisted for strong role fit in Embeddings, MLOps, and Pinecone; fit 84, proof 50, confidence 100, risk 0; Bhubaneswar, Odisha; strong availability signals.</t>
         </is>
       </c>
     </row>
@@ -878,11 +878,11 @@
         <v>44</v>
       </c>
       <c r="C45" s="2">
-        <v>0.5643</v>
+        <v>0.7624</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer with 6.6 yrs; career evidence includes semantic search, embeddings, and faiss; Delhi, Delhi; response rate 0.94; notice 120 days. Concern: long notice period.</t>
+          <t>Recommendation Systems Engineer shortlisted for strong role fit in Embeddings, Hugging Face Transformers, and Learning to Rank; fit 82, proof 45, confidence 92, risk 10; Delhi, Delhi; strong availability signals; good logistics fit; verify Notice period may slow hiring.</t>
         </is>
       </c>
     </row>
@@ -896,11 +896,11 @@
         <v>45</v>
       </c>
       <c r="C46" s="2">
-        <v>0.5544</v>
+        <v>0.7620</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>AI Engineer with 7.2 yrs; career evidence includes embeddings, recommendation system, and ranking; Gurgaon, Haryana; response rate 0.45; notice 30 days. Concern: not marked open to work.</t>
+          <t>AI Engineer shortlisted for strong role fit in BM25 retrieval, Elasticsearch, and Embeddings; fit 94, proof 70, confidence 100, risk 28; Gurgaon, Haryana; good logistics fit; verify Availability is weaker because the candidate is not marked open to work.</t>
         </is>
       </c>
     </row>
@@ -914,11 +914,11 @@
         <v>46</v>
       </c>
       <c r="C47" s="2">
-        <v>0.5445</v>
+        <v>0.7572</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer with 6.8 yrs; career evidence includes embeddings, relevance systems, and recommendation system; Coimbatore, Tamil Nadu; response rate 0.73; notice 60 days.</t>
+          <t>Recommendation Systems Engineer shortlisted for strong role fit in Elasticsearch, Fine-tuning LLMs, and Kubernetes; fit 84, proof 45, confidence 74, risk 0; Coimbatore, Tamil Nadu; strong availability signals; good logistics fit.</t>
         </is>
       </c>
     </row>
@@ -932,11 +932,11 @@
         <v>47</v>
       </c>
       <c r="C48" s="2">
-        <v>0.5346</v>
+        <v>0.7568</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>NLP Engineer with 6.5 yrs; career evidence includes semantic search, faiss, and elasticsearch; Pune, Maharashtra; response rate 0.68; notice 15 days.</t>
+          <t>NLP Engineer shortlisted for strong role fit in Embeddings, Learning to Rank, and LoRA; fit 72, proof 44, confidence 100, risk 0; Pune, Maharashtra; strong availability signals; good logistics fit; verify evaluation methodology or ranking metrics.</t>
         </is>
       </c>
     </row>
@@ -950,11 +950,11 @@
         <v>48</v>
       </c>
       <c r="C49" s="2">
-        <v>0.5247</v>
+        <v>0.7549</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer with 6.9 yrs; career evidence includes embeddings, recommendation system, and ranking; Bangalore, Karnataka; response rate 0.65; notice 45 days.</t>
+          <t>Machine Learning Engineer shortlisted for strong role fit in BentoML, Hugging Face Transformers, and LLM systems; fit 83, proof 47, confidence 78, risk 0; Bangalore, Karnataka; good logistics fit.</t>
         </is>
       </c>
     </row>
@@ -968,11 +968,11 @@
         <v>49</v>
       </c>
       <c r="C50" s="2">
-        <v>0.5148</v>
+        <v>0.7535</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 5.7 yrs; career evidence includes semantic search, embeddings, and faiss; Bangalore, Karnataka; response rate 0.77; notice 90 days.</t>
+          <t>Senior Data Scientist shortlisted for strong role fit in BentoML, FAISS/vector search, and MLflow; fit 79, proof 49, confidence 85, risk 0; Bangalore, Karnataka; strong availability signals; good logistics fit; verify career-backed ranking proof.</t>
         </is>
       </c>
     </row>
@@ -986,11 +986,11 @@
         <v>50</v>
       </c>
       <c r="C51" s="2">
-        <v>0.5049</v>
+        <v>0.7535</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 6.5 yrs; career evidence includes embeddings, recommendation system, and ranking; Noida, Uttar Pradesh; response rate 0.72; notice 120 days. Concern: long notice period.</t>
+          <t>Senior Data Scientist shortlisted for strong role fit in MLflow, Machine Learning, and Milvus; fit 74, proof 49, confidence 98, risk 10; Noida, Uttar Pradesh; strong availability signals; good logistics fit; verify Notice period may slow hiring.</t>
         </is>
       </c>
     </row>
@@ -1004,11 +1004,11 @@
         <v>51</v>
       </c>
       <c r="C52" s="2">
-        <v>0.4951</v>
+        <v>0.7494</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 5.3 yrs; career evidence includes semantic search, faiss, and elasticsearch; Chandigarh, Chandigarh; response rate 0.66; notice 30 days.</t>
+          <t>Senior Data Scientist shortlisted for strong role fit in Elasticsearch, Embeddings, and FastAPI; fit 80, proof 51, confidence 100, risk 0; Chandigarh, Chandigarh; strong availability signals; verify evaluation methodology or ranking metrics.</t>
         </is>
       </c>
     </row>
@@ -1022,11 +1022,11 @@
         <v>52</v>
       </c>
       <c r="C53" s="2">
-        <v>0.4852</v>
+        <v>0.7493</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Applied ML Engineer with 5.2 yrs; career evidence includes semantic search, embeddings, and faiss; Trivandrum, Kerala; response rate 0.52; notice 30 days.</t>
+          <t>Applied ML Engineer shortlisted for strong role fit in BentoML, Elasticsearch, and FAISS/vector search; fit 81, proof 49, confidence 85, risk 0; Trivandrum, Kerala; strong availability signals; verify evaluation methodology or ranking metrics.</t>
         </is>
       </c>
     </row>
@@ -1040,11 +1040,11 @@
         <v>53</v>
       </c>
       <c r="C54" s="2">
-        <v>0.4753</v>
+        <v>0.7480</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 7.6 yrs; career evidence includes embeddings, pinecone, and ranking; Chennai, Tamil Nadu; response rate 0.67; notice 60 days.</t>
+          <t>Senior Data Scientist shortlisted for strong role fit in BentoML, Elasticsearch, and MLOps; fit 81, proof 49, confidence 87, risk 0; Chennai, Tamil Nadu; strong availability signals.</t>
         </is>
       </c>
     </row>
@@ -1058,11 +1058,11 @@
         <v>54</v>
       </c>
       <c r="C55" s="2">
-        <v>0.4654</v>
+        <v>0.7479</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Search Engineer with 7.3 yrs; career evidence includes embeddings, pinecone, and recommendation system; Vizag, Andhra Pradesh; response rate 0.43; notice 90 days.</t>
+          <t>Search Engineer shortlisted for strong role fit in Fine-tuning LLMs, Hugging Face Transformers, and Information Retrieval; fit 84, proof 41, confidence 72, risk 1; Vizag, Andhra Pradesh; good logistics fit.</t>
         </is>
       </c>
     </row>
@@ -1076,11 +1076,11 @@
         <v>55</v>
       </c>
       <c r="C56" s="2">
-        <v>0.4555</v>
+        <v>0.7478</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer with 5.7 yrs; career evidence includes embeddings, pinecone, and relevance systems; Bangalore, Karnataka; response rate 0.58; notice 60 days.</t>
+          <t>Machine Learning Engineer shortlisted for strong role fit in BM25 retrieval, Elasticsearch, and Hugging Face Transformers; fit 79, proof 48, confidence 98, risk 0; Bangalore, Karnataka; strong availability signals; good logistics fit.</t>
         </is>
       </c>
     </row>
@@ -1094,11 +1094,11 @@
         <v>56</v>
       </c>
       <c r="C57" s="2">
-        <v>0.4456</v>
+        <v>0.7474</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>NLP Engineer with 6.6 yrs; career evidence includes embeddings, pinecone, and recommendation system; Vizag, Andhra Pradesh; response rate 0.88; notice 30 days.</t>
+          <t>NLP Engineer shortlisted for strong role fit in Embeddings, FAISS/vector search, and Fine-tuning LLMs; fit 81, proof 43, confidence 86, risk 0; Vizag, Andhra Pradesh; strong availability signals.</t>
         </is>
       </c>
     </row>
@@ -1112,11 +1112,11 @@
         <v>57</v>
       </c>
       <c r="C58" s="2">
-        <v>0.4357</v>
+        <v>0.7433</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer with 5.5 yrs; career evidence includes embeddings, pinecone, and recommendation system; Ahmedabad, Gujarat; response rate 0.56; notice 60 days.</t>
+          <t>Recommendation Systems Engineer shortlisted for strong role fit in BentoML, Embeddings, and FAISS/vector search; fit 77, proof 44, confidence 81, risk 0; Ahmedabad, Gujarat; strong availability signals.</t>
         </is>
       </c>
     </row>
@@ -1130,11 +1130,11 @@
         <v>58</v>
       </c>
       <c r="C59" s="2">
-        <v>0.4258</v>
+        <v>0.7432</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer with 8.0 yrs; career evidence includes search and discovery, relevance systems, and ranking; Noida, Uttar Pradesh; response rate 0.87; notice 30 days.</t>
+          <t>Staff Machine Learning Engineer shortlisted for strong role fit in Information Retrieval Systems, Machine Learning, and Python; fit 82, proof 34, confidence 80, risk 0; Noida, Uttar Pradesh; strong availability signals; good logistics fit.</t>
         </is>
       </c>
     </row>
@@ -1148,11 +1148,11 @@
         <v>59</v>
       </c>
       <c r="C60" s="2">
-        <v>0.4159</v>
+        <v>0.7397</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Search Engineer with 7.6 yrs; career evidence includes semantic search, embeddings, and faiss; Bhubaneswar, Odisha; response rate 0.51; notice 60 days.</t>
+          <t>Search Engineer shortlisted for strong role fit in Elasticsearch, Fine-tuning LLMs, and Hugging Face Transformers; fit 74, proof 38, confidence 76, risk 1; Bhubaneswar, Odisha; strong availability signals; good logistics fit; verify career-backed ranking proof.</t>
         </is>
       </c>
     </row>
@@ -1166,11 +1166,11 @@
         <v>60</v>
       </c>
       <c r="C61" s="2">
-        <v>0.4060</v>
+        <v>0.7378</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer with 6.5 yrs; career evidence includes embeddings, pinecone, and recommendation system; Vizag, Andhra Pradesh; response rate 0.66; notice 15 days.</t>
+          <t>Recommendation Systems Engineer shortlisted for strong role fit in BM25 retrieval, Embeddings, and FAISS/vector search; fit 84, proof 43, confidence 75, risk 1; Vizag, Andhra Pradesh; strong availability signals.</t>
         </is>
       </c>
     </row>
@@ -1184,11 +1184,11 @@
         <v>61</v>
       </c>
       <c r="C62" s="2">
-        <v>0.3961</v>
+        <v>0.7377</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Applied ML Engineer with 6.2 yrs; career evidence includes semantic search, embeddings, and faiss; Ahmedabad, Gujarat; response rate 0.82; notice 45 days.</t>
+          <t>Applied ML Engineer shortlisted for strong role fit in BM25 retrieval, Fine-tuning LLMs, and Learning to Rank; fit 83, proof 46, confidence 86, risk 0; Ahmedabad, Gujarat; strong availability signals.</t>
         </is>
       </c>
     </row>
@@ -1202,11 +1202,11 @@
         <v>62</v>
       </c>
       <c r="C63" s="2">
-        <v>0.3862</v>
+        <v>0.7365</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Senior Applied Scientist with 9.0 yrs; career evidence includes relevance systems, ranking, and evaluation; Kolkata, West Bengal; response rate 0.63; notice 0 days.</t>
+          <t>Senior Applied Scientist shortlisted for strong role fit in BM25 retrieval, BentoML, and Information Retrieval Systems; fit 75, proof 39, confidence 85, risk 0; Kolkata, West Bengal; strong availability signals; good logistics fit.</t>
         </is>
       </c>
     </row>
@@ -1220,11 +1220,11 @@
         <v>63</v>
       </c>
       <c r="C64" s="2">
-        <v>0.3763</v>
+        <v>0.7300</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer with 5.1 yrs; career evidence includes semantic search, faiss, and relevance systems; Kochi, Kerala; response rate 0.70; notice 30 days.</t>
+          <t>Recommendation Systems Engineer shortlisted for strong role fit in BM25 retrieval, Elasticsearch, and FAISS/vector search; fit 79, proof 38, confidence 78, risk 0; Kochi, Kerala; strong availability signals; good logistics fit; verify evaluation methodology or ranking metrics.</t>
         </is>
       </c>
     </row>
@@ -1238,11 +1238,11 @@
         <v>64</v>
       </c>
       <c r="C65" s="2">
-        <v>0.3664</v>
+        <v>0.7289</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer with 7.9 yrs; career evidence includes semantic search, embeddings, and faiss; Noida, Uttar Pradesh; response rate 0.62; notice 30 days.</t>
+          <t>Recommendation Systems Engineer shortlisted for strong role fit in BM25 retrieval, Embeddings, and LLM systems; fit 76, proof 44, confidence 95, risk 0; Noida, Uttar Pradesh; strong availability signals; verify career-backed ranking proof.</t>
         </is>
       </c>
     </row>
@@ -1256,11 +1256,11 @@
         <v>65</v>
       </c>
       <c r="C66" s="2">
-        <v>0.3565</v>
+        <v>0.7278</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Applied ML Engineer with 7.4 yrs; career evidence includes embeddings, recommendation system, and ranking; Coimbatore, Tamil Nadu; response rate 0.53; notice 30 days. Concern: not marked open to work.</t>
+          <t>Applied ML Engineer shortlisted for strong role fit in BentoML, Docker, and FAISS/vector search; fit 86, proof 61, confidence 100, risk 28; Coimbatore, Tamil Nadu; verify Availability is weaker because the candidate is not marked open to work.</t>
         </is>
       </c>
     </row>
@@ -1274,11 +1274,11 @@
         <v>66</v>
       </c>
       <c r="C67" s="2">
-        <v>0.3466</v>
+        <v>0.7244</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Applied ML Engineer with 5.0 yrs; career evidence includes embeddings, recommendation system, and ranking; Hyderabad, Telangana; response rate 0.84; notice 120 days. Concern: long notice period.</t>
+          <t>Applied ML Engineer shortlisted for strong role fit in BM25 retrieval, BentoML, and Hugging Face Transformers; fit 80, proof 44, confidence 87, risk 10; Hyderabad, Telangana; strong availability signals; good logistics fit; verify Notice period may slow hiring.</t>
         </is>
       </c>
     </row>
@@ -1292,11 +1292,11 @@
         <v>67</v>
       </c>
       <c r="C68" s="2">
-        <v>0.3367</v>
+        <v>0.7230</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer with 7.1 yrs; career evidence includes semantic search, faiss, and ranking; Noida, Uttar Pradesh; response rate 0.47; notice 30 days.</t>
+          <t>Machine Learning Engineer shortlisted for strong role fit in Fine-tuning LLMs, Hugging Face Transformers, and MLOps; fit 70, proof 42, confidence 81, risk 1; Noida, Uttar Pradesh; strong availability signals; good logistics fit; verify career-backed retrieval proof.</t>
         </is>
       </c>
     </row>
@@ -1310,11 +1310,11 @@
         <v>68</v>
       </c>
       <c r="C69" s="2">
-        <v>0.3268</v>
+        <v>0.7214</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>AI Engineer with 5.8 yrs; career evidence includes semantic search, embeddings, and faiss; Chennai, Tamil Nadu; response rate 0.69; notice 90 days.</t>
+          <t>AI Engineer shortlisted for strong role fit in Hugging Face Transformers, MLOps, and Machine Learning; fit 72, proof 45, confidence 80, risk 0; Chennai, Tamil Nadu; good logistics fit; verify career-backed ranking proof.</t>
         </is>
       </c>
     </row>
@@ -1328,11 +1328,11 @@
         <v>69</v>
       </c>
       <c r="C70" s="2">
-        <v>0.3169</v>
+        <v>0.7212</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer with 4.8 yrs; career evidence includes semantic search, embeddings, and faiss; Chennai, Tamil Nadu; response rate 0.52; notice 90 days.</t>
+          <t>Recommendation Systems Engineer shortlisted for strong role fit in BentoML, Embeddings, and FAISS/vector search; fit 78, proof 44, confidence 72, risk 0; Chennai, Tamil Nadu; strong availability signals; good logistics fit.</t>
         </is>
       </c>
     </row>
@@ -1346,11 +1346,11 @@
         <v>70</v>
       </c>
       <c r="C71" s="2">
-        <v>0.3070</v>
+        <v>0.7160</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer with 6.0 yrs; career evidence includes semantic search, faiss, and elasticsearch; Trivandrum, Kerala; response rate 0.90; notice 30 days.</t>
+          <t>Recommendation Systems Engineer shortlisted for strong role fit in Embeddings, FAISS/vector search, and Hugging Face Transformers; fit 80, proof 36, confidence 76, risk 0; Trivandrum, Kerala; strong availability signals; verify career-backed ranking proof.</t>
         </is>
       </c>
     </row>
@@ -1364,11 +1364,11 @@
         <v>71</v>
       </c>
       <c r="C72" s="2">
-        <v>0.2971</v>
+        <v>0.7158</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Applied ML Engineer with 5.5 yrs; career evidence includes embeddings, pinecone, and recommendation system; Chandigarh, Chandigarh; response rate 0.77; notice 90 days.</t>
+          <t>Applied ML Engineer shortlisted for strong role fit in BentoML, Elasticsearch, and Information Retrieval; fit 69, proof 42, confidence 79, risk 0; Chandigarh, Chandigarh; strong availability signals; verify career-backed ranking proof.</t>
         </is>
       </c>
     </row>
@@ -1382,11 +1382,11 @@
         <v>72</v>
       </c>
       <c r="C73" s="2">
-        <v>0.2872</v>
+        <v>0.7146</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>NLP Engineer with 5.4 yrs; career evidence includes semantic search, embeddings, and faiss; Chandigarh, Chandigarh; response rate 0.83; notice 90 days.</t>
+          <t>NLP Engineer shortlisted for strong role fit in Learning to Rank, LoRA, and Machine Learning; fit 71, proof 37, confidence 78, risk 0; Chandigarh, Chandigarh; strong availability signals; good logistics fit.</t>
         </is>
       </c>
     </row>
@@ -1400,11 +1400,11 @@
         <v>73</v>
       </c>
       <c r="C74" s="2">
-        <v>0.2773</v>
+        <v>0.7140</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer with 6.9 yrs; career evidence includes embeddings, pinecone, and ranking; Bangalore, Karnataka; response rate 0.50; notice 15 days.</t>
+          <t>Machine Learning Engineer shortlisted for strong role fit in BM25 retrieval, Elasticsearch, and LLM systems; fit 73, proof 33, confidence 64, risk 0; Bangalore, Karnataka; strong availability signals; good logistics fit; verify career-backed ranking proof.</t>
         </is>
       </c>
     </row>
@@ -1418,11 +1418,11 @@
         <v>74</v>
       </c>
       <c r="C75" s="2">
-        <v>0.2674</v>
+        <v>0.7109</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Applied ML Engineer with 5.7 yrs; career evidence includes semantic search, embeddings, and faiss; Mumbai, Maharashtra; response rate 0.51; notice 90 days.</t>
+          <t>Applied ML Engineer shortlisted for strong role fit in BM25 retrieval, FAISS/vector search, and Fine-tuning LLMs; fit 77, proof 45, confidence 87, risk 1; Mumbai, Maharashtra; good logistics fit.</t>
         </is>
       </c>
     </row>
@@ -1436,11 +1436,11 @@
         <v>75</v>
       </c>
       <c r="C76" s="2">
-        <v>0.2575</v>
+        <v>0.7096</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>NLP Engineer with 6.8 yrs; career evidence includes semantic search, embeddings, and faiss; Indore, Madhya Pradesh; response rate 0.83; notice 60 days. Concern: not marked open to work.</t>
+          <t>NLP Engineer shortlisted for strong role fit in Elasticsearch, Hugging Face Transformers, and Machine Learning; fit 88, proof 56, confidence 81, risk 28; Indore, Madhya Pradesh; good logistics fit; verify Availability is weaker because the candidate is not marked open to work.</t>
         </is>
       </c>
     </row>
@@ -1454,11 +1454,11 @@
         <v>76</v>
       </c>
       <c r="C77" s="2">
-        <v>0.2476</v>
+        <v>0.7082</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>AI Engineer with 7.3 yrs; career evidence includes semantic search, embeddings, and faiss; Kochi, Kerala; response rate 0.78; notice 30 days.</t>
+          <t>AI Engineer shortlisted for strong role fit in BM25 retrieval, Hugging Face Transformers, and Information Retrieval; fit 74, proof 37, confidence 77, risk 0; Kochi, Kerala; strong availability signals; good logistics fit; verify evaluation methodology or ranking metrics.</t>
         </is>
       </c>
     </row>
@@ -1472,11 +1472,11 @@
         <v>77</v>
       </c>
       <c r="C78" s="2">
-        <v>0.2377</v>
+        <v>0.7065</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer with 15.2 yrs; career evidence includes semantic search, faiss, and elasticsearch; Kolkata, West Bengal; response rate 0.73; notice 30 days.</t>
+          <t>Recommendation Systems Engineer shortlisted for strong role fit in BM25 retrieval, LLM systems, and Learning to Rank; fit 81, proof 61, confidence 100, risk 17; Kolkata, West Bengal; strong availability signals; good logistics fit.</t>
         </is>
       </c>
     </row>
@@ -1490,11 +1490,11 @@
         <v>78</v>
       </c>
       <c r="C79" s="2">
-        <v>0.2278</v>
+        <v>0.7063</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Search Engineer with 4.2 yrs; career evidence includes semantic search, embeddings, and faiss; Mumbai, Maharashtra; response rate 0.48; notice 15 days.</t>
+          <t>Search Engineer shortlisted for strong role fit in Airflow, BentoML, and FAISS/vector search; fit 73, proof 42, confidence 72, risk 0; Mumbai, Maharashtra; strong availability signals.</t>
         </is>
       </c>
     </row>
@@ -1508,11 +1508,11 @@
         <v>79</v>
       </c>
       <c r="C80" s="2">
-        <v>0.2179</v>
+        <v>0.7007</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer with 3.0 yrs; career evidence includes semantic search, embeddings, and faiss; Trivandrum, Kerala; response rate 0.57; notice 90 days.</t>
+          <t>Machine Learning Engineer shortlisted for strong role fit in FAISS/vector search, Fine-tuning LLMs, and Information Retrieval; fit 70, proof 55, confidence 94, risk 0; Trivandrum, Kerala; strong availability signals; good logistics fit.</t>
         </is>
       </c>
     </row>
@@ -1526,11 +1526,11 @@
         <v>80</v>
       </c>
       <c r="C81" s="2">
-        <v>0.2080</v>
+        <v>0.7002</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer with 7.2 yrs; career evidence includes semantic search, faiss, and elasticsearch; Kochi, Kerala; response rate 0.60; notice 120 days. Concern: long notice period.</t>
+          <t>Machine Learning Engineer shortlisted for strong role fit in BM25 retrieval, Embeddings, and FAISS/vector search; fit 79, proof 47, confidence 98, risk 10; Kochi, Kerala; good logistics fit; verify Notice period may slow hiring.</t>
         </is>
       </c>
     </row>
@@ -1544,11 +1544,11 @@
         <v>81</v>
       </c>
       <c r="C82" s="2">
-        <v>0.1981</v>
+        <v>0.6985</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer with 6.5 yrs; career evidence includes embeddings, pinecone, and recommendation system; Pune, Maharashtra; response rate 0.79; notice 30 days.</t>
+          <t>Recommendation Systems Engineer shortlisted for strong role fit in Fine-tuning LLMs, Learning to Rank, and LoRA; fit 72, proof 30, confidence 71, risk 10; Pune, Maharashtra; strong availability signals; good logistics fit; verify career-backed ranking proof.</t>
         </is>
       </c>
     </row>
@@ -1562,11 +1562,11 @@
         <v>82</v>
       </c>
       <c r="C83" s="2">
-        <v>0.1882</v>
+        <v>0.6963</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>NLP Engineer with 7.7 yrs; career evidence includes embeddings, relevance systems, and recommendation system; Ahmedabad, Gujarat; response rate 0.42; notice 90 days. Concern: not marked open to work.</t>
+          <t>NLP Engineer shortlisted for strong role fit in BM25 retrieval, Embeddings, and Information Retrieval; fit 78, proof 60, confidence 100, risk 28; Ahmedabad, Gujarat; good logistics fit; verify Availability is weaker because the candidate is not marked open to work.</t>
         </is>
       </c>
     </row>
@@ -1580,11 +1580,11 @@
         <v>83</v>
       </c>
       <c r="C84" s="2">
-        <v>0.1783</v>
+        <v>0.6960</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer with 5.9 yrs; career evidence includes relevance systems, ranking, and learning-to-rank; Delhi, Delhi; response rate 0.63; notice 15 days.</t>
+          <t>Recommendation Systems Engineer shortlisted for strong role fit in BM25 retrieval, Embeddings, and FAISS/vector search; fit 72, proof 33, confidence 61, risk 0; Delhi, Delhi; strong availability signals; good logistics fit; verify evaluation methodology or ranking metrics.</t>
         </is>
       </c>
     </row>
@@ -1598,11 +1598,11 @@
         <v>84</v>
       </c>
       <c r="C85" s="2">
-        <v>0.1684</v>
+        <v>0.6902</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>NLP Engineer with 7.9 yrs; career evidence includes embeddings, relevance systems, and recommendation system; Jaipur, Rajasthan; response rate 0.63; notice 120 days. Concern: long notice period.</t>
+          <t>NLP Engineer shortlisted for strong role fit in Elasticsearch, FAISS/vector search, and Hugging Face Transformers; fit 80, proof 44, confidence 73, risk 11; Jaipur, Rajasthan; strong availability signals; good logistics fit; verify Notice period may slow hiring.</t>
         </is>
       </c>
     </row>
@@ -1616,11 +1616,11 @@
         <v>85</v>
       </c>
       <c r="C86" s="2">
-        <v>0.1585</v>
+        <v>0.6888</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>NLP Engineer with 2.8 yrs; career evidence includes embeddings, pinecone, and ranking; Chennai, Tamil Nadu; response rate 0.87; notice 90 days.</t>
+          <t>NLP Engineer shortlisted for strong role fit in BM25 retrieval, LLM systems, and Milvus; fit 71, proof 57, confidence 100, risk 0; Chennai, Tamil Nadu; strong availability signals.</t>
         </is>
       </c>
     </row>
@@ -1634,11 +1634,11 @@
         <v>86</v>
       </c>
       <c r="C87" s="2">
-        <v>0.1486</v>
+        <v>0.6881</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Lead AI Engineer with 6.4 yrs; career evidence includes search and discovery, matching layer, and relevance systems; Delhi, Delhi; response rate 0.86; notice 0 days. Concern: not marked open to work.</t>
+          <t>Lead AI Engineer shortlisted for strong role fit in Elasticsearch, Information Retrieval Systems, and LoRA; fit 90, proof 48, confidence 100, risk 29; Delhi, Delhi; verify Availability is weaker because the candidate is not marked open to work.</t>
         </is>
       </c>
     </row>
@@ -1652,11 +1652,11 @@
         <v>87</v>
       </c>
       <c r="C88" s="2">
-        <v>0.1387</v>
+        <v>0.6880</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>AI Engineer with 5.7 yrs; career evidence includes embeddings, recommendation system, and ranking; Trivandrum, Kerala; response rate 0.94; notice 30 days. Concern: not marked open to work.</t>
+          <t>AI Engineer shortlisted for strong role fit in BM25 retrieval, Information Retrieval, and LoRA; fit 81, proof 53, confidence 100, risk 28; Trivandrum, Kerala; strong availability signals; verify Availability is weaker because the candidate is not marked open to work.</t>
         </is>
       </c>
     </row>
@@ -1670,11 +1670,11 @@
         <v>88</v>
       </c>
       <c r="C89" s="2">
-        <v>0.1288</v>
+        <v>0.6870</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 5.3 yrs; career evidence includes embeddings, recommendation system, and ranking; Indore, Madhya Pradesh; response rate 0.55; notice 45 days.</t>
+          <t>Senior Data Scientist shortlisted for strong role fit in Elasticsearch, Fine-tuning LLMs, and MLOps; fit 69, proof 42, confidence 82, risk 1; Indore, Madhya Pradesh; strong availability signals.</t>
         </is>
       </c>
     </row>
@@ -1688,11 +1688,11 @@
         <v>89</v>
       </c>
       <c r="C90" s="2">
-        <v>0.1189</v>
+        <v>0.6855</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>AI Engineer with 6.4 yrs; career evidence includes semantic search, embeddings, and faiss; Jaipur, Rajasthan; response rate 0.86; notice 15 days. Concern: not marked open to work.</t>
+          <t>AI Engineer shortlisted for strong role fit in Elasticsearch, FAISS/vector search, and Recommendation Systems; fit 86, proof 55, confidence 100, risk 29; Jaipur, Rajasthan; good logistics fit; verify Availability is weaker because the candidate is not marked open to work.</t>
         </is>
       </c>
     </row>
@@ -1706,11 +1706,11 @@
         <v>90</v>
       </c>
       <c r="C91" s="2">
-        <v>0.1090</v>
+        <v>0.6854</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>AI Engineer with 4.9 yrs; career evidence includes embeddings, recommendation system, and ranking; Hyderabad, Telangana; response rate 0.78; notice 90 days.</t>
+          <t>AI Engineer shortlisted for strong role fit in Elasticsearch, Embeddings, and FastAPI; fit 64, proof 39, confidence 89, risk 0; Hyderabad, Telangana; strong availability signals; good logistics fit.</t>
         </is>
       </c>
     </row>
@@ -1724,11 +1724,11 @@
         <v>91</v>
       </c>
       <c r="C92" s="2">
-        <v>0.0991</v>
+        <v>0.6851</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 4.3 yrs; career evidence includes embeddings, pinecone, and relevance systems; Chennai, Tamil Nadu; response rate 0.46; notice 60 days.</t>
+          <t>Senior Data Scientist shortlisted for strong role fit in BM25 retrieval, FAISS/vector search, and LoRA; fit 70, proof 49, confidence 85, risk 1; Chennai, Tamil Nadu; strong availability signals; good logistics fit; verify evaluation methodology or ranking metrics.</t>
         </is>
       </c>
     </row>
@@ -1742,11 +1742,11 @@
         <v>92</v>
       </c>
       <c r="C93" s="2">
-        <v>0.0892</v>
+        <v>0.6825</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer with 4.5 yrs; career evidence includes semantic search, embeddings, and faiss; Noida, Uttar Pradesh; response rate 0.54; notice 45 days.</t>
+          <t>Machine Learning Engineer shortlisted for strong role fit in Elasticsearch, Embeddings, and MLOps; fit 71, proof 44, confidence 84, risk 1; Noida, Uttar Pradesh; strong availability signals; good logistics fit.</t>
         </is>
       </c>
     </row>
@@ -1760,11 +1760,11 @@
         <v>93</v>
       </c>
       <c r="C94" s="2">
-        <v>0.0793</v>
+        <v>0.6825</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Senior Applied Scientist with 5.4 yrs; career evidence includes relevance systems, ranking, and A/B testing; Indore, Madhya Pradesh; response rate 0.78; notice 45 days.</t>
+          <t>Senior Applied Scientist shortlisted for strong role fit in Information Retrieval Systems, Machine Learning, and Milvus; fit 74, proof 28, confidence 76, risk 0; Indore, Madhya Pradesh; strong availability signals.</t>
         </is>
       </c>
     </row>
@@ -1778,11 +1778,11 @@
         <v>94</v>
       </c>
       <c r="C95" s="2">
-        <v>0.0694</v>
+        <v>0.6794</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Senior Machine Learning Engineer with 7.9 yrs; career evidence includes matching layer, ranking, and explicit modeling; Bangalore, Karnataka; response rate 0.61; notice 45 days.</t>
+          <t>Senior Machine Learning Engineer shortlisted for strong role fit in Information Retrieval Systems, Machine Learning, and OpenSearch; fit 79, proof 28, confidence 73, risk 0; Bangalore, Karnataka; strong availability signals; good logistics fit; verify evaluation methodology or ranking metrics.</t>
         </is>
       </c>
     </row>
@@ -1796,11 +1796,11 @@
         <v>95</v>
       </c>
       <c r="C96" s="2">
-        <v>0.0595</v>
+        <v>0.6771</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Search Engineer with 5.1 yrs; career evidence includes embeddings, pinecone, and ranking; Kolkata, West Bengal; response rate 0.80; notice 45 days.</t>
+          <t>Search Engineer shortlisted for strong role fit in BentoML, Elasticsearch, and Hugging Face Transformers; fit 71, proof 32, confidence 59, risk 10; Kolkata, West Bengal; strong availability signals; verify career-backed ranking proof.</t>
         </is>
       </c>
     </row>
@@ -1814,11 +1814,11 @@
         <v>96</v>
       </c>
       <c r="C97" s="2">
-        <v>0.0496</v>
+        <v>0.6770</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 6.6 yrs; career evidence includes semantic search, embeddings, and faiss; Coimbatore, Tamil Nadu; response rate 0.57; notice 60 days. Concern: not marked open to work.</t>
+          <t>Senior Data Scientist shortlisted for strong role fit in BentoML, Embeddings, and Hugging Face Transformers; fit 80, proof 54, confidence 100, risk 28; Coimbatore, Tamil Nadu; good logistics fit; verify Availability is weaker because the candidate is not marked open to work.</t>
         </is>
       </c>
     </row>
@@ -1832,11 +1832,11 @@
         <v>97</v>
       </c>
       <c r="C98" s="2">
-        <v>0.0397</v>
+        <v>0.6767</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer with 5.7 yrs; career evidence includes ranking, evaluation, and A/B testing; Gurgaon, Haryana; response rate 0.92; notice 60 days.</t>
+          <t>Machine Learning Engineer shortlisted for strong role fit in Elasticsearch, Embeddings, and Kubernetes; fit 65, proof 33, confidence 74, risk 0; Gurgaon, Haryana; strong availability signals; good logistics fit; verify career-backed retrieval proof.</t>
         </is>
       </c>
     </row>
@@ -1850,11 +1850,11 @@
         <v>98</v>
       </c>
       <c r="C99" s="2">
-        <v>0.0298</v>
+        <v>0.6762</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Applied ML Engineer with 6.8 yrs; career evidence includes semantic search, faiss, and elasticsearch; Chennai, Tamil Nadu; response rate 0.41; notice 30 days. Concern: not marked open to work.</t>
+          <t>Applied ML Engineer shortlisted for strong role fit in FastAPI, Hugging Face Transformers, and Learning to Rank; fit 78, proof 47, confidence 100, risk 28; Chennai, Tamil Nadu; strong availability signals; verify Availability is weaker because the candidate is not marked open to work.</t>
         </is>
       </c>
     </row>
@@ -1868,11 +1868,11 @@
         <v>99</v>
       </c>
       <c r="C100" s="2">
-        <v>0.0199</v>
+        <v>0.6760</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>NLP Engineer with 7.4 yrs; career evidence includes semantic search, faiss, and elasticsearch; Hyderabad, Telangana; response rate 0.65; notice 120 days. Concern: long notice period.</t>
+          <t>NLP Engineer shortlisted for strong role fit in FAISS/vector search, Learning to Rank, and MLOps; fit 69, proof 42, confidence 90, risk 10; Hyderabad, Telangana; strong availability signals; good logistics fit; verify Notice period may slow hiring.</t>
         </is>
       </c>
     </row>
@@ -1886,11 +1886,11 @@
         <v>100</v>
       </c>
       <c r="C101" s="2">
-        <v>0.0100</v>
+        <v>0.6702</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>AI Engineer with 5.4 yrs; career evidence includes embeddings, pinecone, and recommendation system; Delhi, Delhi; response rate 0.65; notice 90 days.</t>
+          <t>AI Engineer shortlisted for strong role fit in BM25 retrieval, BentoML, and Embeddings; fit 71, proof 35, confidence 64, risk 0; Delhi, Delhi; good logistics fit; verify career-backed ranking proof.</t>
         </is>
       </c>
     </row>

</xml_diff>